<commit_message>
refactor(tasks): introduce DTO boundary for task service
</commit_message>
<xml_diff>
--- a/docs/Lifelikegame_Phase_Progress_Tracker_CN.xlsx
+++ b/docs/Lifelikegame_Phase_Progress_Tracker_CN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\folder\projects\lifelikegame\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB7FBD6E-734C-49F2-A87C-82CA5272B855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292B06E0-057A-441D-8D07-8EF13183BB1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4730,10 +4730,10 @@
         <v>7</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="H6" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>8</v>
@@ -4774,10 +4774,10 @@
         <v>11</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="H7" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>8</v>

</xml_diff>